<commit_message>
test: align TC-003 with operator home
</commit_message>
<xml_diff>
--- a/qa-docs/07-test-cases.xlsx
+++ b/qa-docs/07-test-cases.xlsx
@@ -16910,7 +16910,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="122.8" customHeight="1">
+    <row r="4" ht="96.39999999999999" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
           <t>TC-003</t>
@@ -16923,13 +16923,13 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>/dashboard/calls</t>
+          <t>/dashboard/home</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
           <t>Вход оператора с верными логином и паролем
-Проверяем вход оператора и его стартовый экран. ВНИМАНИЕ: по коду фронтенда оператора после входа ведут на «Звонки» (/dashboard/calls), а не на «Рабочий стол», как написано в старой документации. Код — источник правды.</t>
+Проверяем вход оператора и его стартовый экран. Уточнено по факту 28.07.2026: корректный стартовый экран оператора — «Рабочий стол» (/dashboard/home).</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
@@ -16947,7 +16947,7 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Вход выполнен. Открывается раздел «Звонки» (адрес /dashboard/calls) — таблица лидов. В меню слева: «Рабочий стол», «Режим звонков», «Звонки», «Рабочее время».</t>
+          <t>Вход выполнен. Открывается раздел «Рабочий стол» (адрес /dashboard/home): видны блок «Последние звонки» и кнопка «Начать звонок». В меню слева: «Рабочий стол», «Режим звонков», «Звонки», «Рабочее время».</t>
         </is>
       </c>
       <c r="H4" s="20" t="inlineStr">

</xml_diff>